<commit_message>
Remove filtros; comprovantes do Drive em pastas Ano/Mes; renomeia Alelo para Santander - Soma (tela/PDF/Excel); cache v20
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -81,10 +81,10 @@
     <t>SUBTOTAL DESPESAS PARA REEMBOLSO:</t>
   </si>
   <si>
-    <t>DESPESAS CARTÃO ALELO</t>
+    <t>DESPESAS CARTÃO SANTANDER - SOMA</t>
   </si>
   <si>
-    <t>SUBTOTAL DESPESAS PARA CARTÃO ALELO:</t>
+    <t>SUBTOTAL DESPESAS CARTÃO SANTANDER - SOMA:</t>
   </si>
   <si>
     <t>TOTAL DOS GASTOS</t>

</xml_diff>